<commit_message>
update the excel file
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TA38804\Downloads\DOCs\Documents\ALL PFE Projects\dashboard-static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2580431-0447-4CD2-99DA-66B10B278620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1553A5B2-8A6A-459F-A1D2-A6A9DFB4F754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
     <sheet name="Repartition Arrivee Usine" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'integration Usine'!$B$1:$E$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'integration Usine'!$B$1:$E$159</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="82">
   <si>
     <t>Des arrivees Non diplomes</t>
   </si>
@@ -263,13 +263,31 @@
     <t>Apprentis O2X</t>
   </si>
   <si>
-    <t>APPRENTIS  EMB</t>
-  </si>
-  <si>
     <t>APPRENTIS O2X</t>
   </si>
   <si>
     <t xml:space="preserve">Moteur Apprentis </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ferrage non diplomé </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NON </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEI APPRENTIS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">non </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOT </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FER </t>
   </si>
 </sst>
 </file>
@@ -585,7 +603,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -598,6 +615,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -932,7 +950,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:F147"/>
+  <dimension ref="B1:F159"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="15" customWidth="1"/>
@@ -2494,7 +2512,7 @@
     </row>
     <row r="96" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B96" s="15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C96" s="12">
         <v>3</v>
@@ -2646,19 +2664,19 @@
       </c>
     </row>
     <row r="105" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B105" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="C105" s="37">
+      <c r="B105" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="C105" s="36">
         <v>28</v>
       </c>
-      <c r="D105" s="38">
+      <c r="D105" s="37">
         <v>46241</v>
       </c>
-      <c r="E105" s="39">
+      <c r="E105" s="38">
         <v>46255</v>
       </c>
-      <c r="F105" s="37" t="s">
+      <c r="F105" s="36" t="s">
         <v>29</v>
       </c>
     </row>
@@ -2783,7 +2801,7 @@
     </row>
     <row r="113" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B113" s="15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C113" s="15">
         <v>4</v>
@@ -2834,7 +2852,7 @@
     </row>
     <row r="116" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B116" s="15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C116" s="12">
         <v>4</v>
@@ -2902,7 +2920,7 @@
     </row>
     <row r="120" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B120" s="12" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="C120" s="12">
         <v>1</v>
@@ -3021,7 +3039,7 @@
     </row>
     <row r="127" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B127" s="15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C127" s="12">
         <v>1</v>
@@ -3157,7 +3175,7 @@
     </row>
     <row r="135" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B135" s="12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C135" s="12">
         <v>1</v>
@@ -3242,7 +3260,7 @@
       <c r="D140" s="24">
         <v>46273</v>
       </c>
-      <c r="E140" s="36">
+      <c r="E140" s="35">
         <v>46288</v>
       </c>
       <c r="F140" s="12" t="s">
@@ -3259,7 +3277,7 @@
       <c r="D141" s="24">
         <v>46273</v>
       </c>
-      <c r="E141" s="36">
+      <c r="E141" s="35">
         <v>46288</v>
       </c>
       <c r="F141" s="12" t="s">
@@ -3276,7 +3294,7 @@
       <c r="D142" s="24">
         <v>46273</v>
       </c>
-      <c r="E142" s="36">
+      <c r="E142" s="35">
         <v>46288</v>
       </c>
       <c r="F142" s="12" t="s">
@@ -3293,7 +3311,7 @@
       <c r="D143" s="24">
         <v>46273</v>
       </c>
-      <c r="E143" s="36">
+      <c r="E143" s="35">
         <v>46288</v>
       </c>
       <c r="F143" s="12" t="s">
@@ -3310,24 +3328,270 @@
       <c r="D144" s="24">
         <v>46273</v>
       </c>
-      <c r="E144" s="36">
+      <c r="E144" s="35">
         <v>46288</v>
       </c>
       <c r="F144" s="12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B145"/>
-    </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B146"/>
-    </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B147"/>
+    <row r="145" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B145" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C145" s="12">
+        <v>89</v>
+      </c>
+      <c r="D145" s="24">
+        <v>46274</v>
+      </c>
+      <c r="E145" s="35">
+        <v>46289</v>
+      </c>
+      <c r="F145" s="12" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="146" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B146" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C146" s="12">
+        <v>37</v>
+      </c>
+      <c r="D146" s="24">
+        <v>46279</v>
+      </c>
+      <c r="E146" s="24">
+        <v>46294</v>
+      </c>
+      <c r="F146" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="147" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B147" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C147" s="12">
+        <v>20</v>
+      </c>
+      <c r="D147" s="24">
+        <v>46279</v>
+      </c>
+      <c r="E147" s="24">
+        <v>46294</v>
+      </c>
+      <c r="F147" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="148" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B148" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C148" s="12">
+        <v>17</v>
+      </c>
+      <c r="D148" s="24">
+        <v>46279</v>
+      </c>
+      <c r="E148" s="24">
+        <v>46294</v>
+      </c>
+      <c r="F148" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="149" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B149" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C149" s="12">
+        <v>26</v>
+      </c>
+      <c r="D149" s="24">
+        <v>46279</v>
+      </c>
+      <c r="E149" s="24">
+        <v>46294</v>
+      </c>
+      <c r="F149" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="150" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B150" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C150" s="12">
+        <v>1</v>
+      </c>
+      <c r="D150" s="24">
+        <v>46279</v>
+      </c>
+      <c r="E150" s="24">
+        <v>46294</v>
+      </c>
+      <c r="F150" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="151" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B151" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C151" s="12">
+        <v>1</v>
+      </c>
+      <c r="D151" s="24">
+        <v>46279</v>
+      </c>
+      <c r="E151" s="24">
+        <v>46294</v>
+      </c>
+      <c r="F151" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="152" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B152" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C152" s="12">
+        <v>1</v>
+      </c>
+      <c r="D152" s="24">
+        <v>46279</v>
+      </c>
+      <c r="E152" s="24">
+        <v>46294</v>
+      </c>
+      <c r="F152" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="153" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B153" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C153" s="12">
+        <v>71</v>
+      </c>
+      <c r="D153" s="24">
+        <v>46280</v>
+      </c>
+      <c r="E153" s="24">
+        <v>46294</v>
+      </c>
+      <c r="F153" s="12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="154" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B154" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C154" s="12">
+        <v>14</v>
+      </c>
+      <c r="D154" s="24">
+        <v>46282</v>
+      </c>
+      <c r="E154" s="24">
+        <v>46295</v>
+      </c>
+      <c r="F154" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="155" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B155" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C155" s="15">
+        <v>40</v>
+      </c>
+      <c r="D155" s="24">
+        <v>46282</v>
+      </c>
+      <c r="E155" s="24">
+        <v>46295</v>
+      </c>
+      <c r="F155" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="156" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B156" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C156" s="15">
+        <v>27</v>
+      </c>
+      <c r="D156" s="24">
+        <v>46282</v>
+      </c>
+      <c r="E156" s="24">
+        <v>46295</v>
+      </c>
+      <c r="F156" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="157" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B157" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C157" s="15">
+        <v>11</v>
+      </c>
+      <c r="D157" s="24">
+        <v>46282</v>
+      </c>
+      <c r="E157" s="24">
+        <v>46295</v>
+      </c>
+      <c r="F157" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="158" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B158" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C158" s="15">
+        <v>24</v>
+      </c>
+      <c r="D158" s="24">
+        <v>46282</v>
+      </c>
+      <c r="E158" s="24">
+        <v>46295</v>
+      </c>
+      <c r="F158" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="159" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B159" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C159" s="15">
+        <v>20</v>
+      </c>
+      <c r="D159" s="24">
+        <v>46282</v>
+      </c>
+      <c r="E159" s="24">
+        <v>46295</v>
+      </c>
+      <c r="F159" s="12" t="s">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:E144" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="B1:E159" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3342,20 +3606,20 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="35"/>
-      <c r="J4" s="35"/>
-      <c r="K4" s="35"/>
-      <c r="L4" s="35"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+      <c r="L4" s="39"/>
     </row>
     <row r="5" spans="1:12" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G5" s="34"/>

</xml_diff>

<commit_message>
update the dashboard values
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\user\TB45426\Documents\ALL project\dashboard-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A47B959-B843-46F6-A959-0075490AD7EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3C3017E-3AA6-47F3-B7BA-4314A614B7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="integration Usine" sheetId="1" r:id="rId1"/>
@@ -22,14 +22,30 @@
     <sheet name="Repartition Arrivee Usine" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'integration Usine'!$B$1:$E$172</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'integration Usine'!$B$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="88">
   <si>
     <t>Des arrivees Non diplomes</t>
   </si>
@@ -278,13 +294,28 @@
   </si>
   <si>
     <t xml:space="preserve">USINAGE </t>
+  </si>
+  <si>
+    <t>Make Batterie</t>
+  </si>
+  <si>
+    <t>S41</t>
+  </si>
+  <si>
+    <t>S42</t>
+  </si>
+  <si>
+    <t>S43</t>
+  </si>
+  <si>
+    <t>S44</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -325,8 +356,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -354,6 +399,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -499,7 +550,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -606,6 +657,20 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -940,7 +1005,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:F172"/>
+  <dimension ref="B1:F207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="15" customWidth="1"/>
@@ -3801,8 +3866,478 @@
         <v>25</v>
       </c>
     </row>
+    <row r="173" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B173" s="44" t="s">
+        <v>66</v>
+      </c>
+      <c r="C173" s="44">
+        <v>15</v>
+      </c>
+      <c r="D173" s="45">
+        <v>46308</v>
+      </c>
+      <c r="E173" s="45">
+        <f>D173+15</f>
+        <v>46323</v>
+      </c>
+      <c r="F173" s="44"/>
+    </row>
+    <row r="174" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B174" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C174" s="12">
+        <v>8</v>
+      </c>
+      <c r="D174" s="24">
+        <v>46322</v>
+      </c>
+      <c r="E174" s="24">
+        <f t="shared" ref="E174:E197" si="0">D174+15</f>
+        <v>46337</v>
+      </c>
+      <c r="F174" s="12"/>
+    </row>
+    <row r="175" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B175" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C175" s="12">
+        <v>20</v>
+      </c>
+      <c r="D175" s="24">
+        <v>46296</v>
+      </c>
+      <c r="E175" s="24">
+        <f t="shared" si="0"/>
+        <v>46311</v>
+      </c>
+      <c r="F175" s="12"/>
+    </row>
+    <row r="176" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B176" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C176" s="12">
+        <v>40</v>
+      </c>
+      <c r="D176" s="24">
+        <v>46309</v>
+      </c>
+      <c r="E176" s="24">
+        <f t="shared" si="0"/>
+        <v>46324</v>
+      </c>
+      <c r="F176" s="12"/>
+    </row>
+    <row r="177" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B177" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C177" s="12">
+        <v>21</v>
+      </c>
+      <c r="D177" s="24">
+        <v>46316</v>
+      </c>
+      <c r="E177" s="24">
+        <f t="shared" si="0"/>
+        <v>46331</v>
+      </c>
+      <c r="F177" s="12"/>
+    </row>
+    <row r="178" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B178" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C178" s="12">
+        <v>1</v>
+      </c>
+      <c r="D178" s="24">
+        <v>46301</v>
+      </c>
+      <c r="E178" s="24">
+        <f t="shared" si="0"/>
+        <v>46316</v>
+      </c>
+      <c r="F178" s="12"/>
+    </row>
+    <row r="179" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B179" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C179" s="12">
+        <v>26</v>
+      </c>
+      <c r="D179" s="24">
+        <v>46305</v>
+      </c>
+      <c r="E179" s="24">
+        <f t="shared" si="0"/>
+        <v>46320</v>
+      </c>
+      <c r="F179" s="12"/>
+    </row>
+    <row r="180" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B180" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C180" s="12">
+        <v>93</v>
+      </c>
+      <c r="D180" s="24">
+        <v>46301</v>
+      </c>
+      <c r="E180" s="24">
+        <f t="shared" si="0"/>
+        <v>46316</v>
+      </c>
+      <c r="F180" s="12"/>
+    </row>
+    <row r="181" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B181" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C181" s="12">
+        <v>1</v>
+      </c>
+      <c r="D181" s="24">
+        <v>46308</v>
+      </c>
+      <c r="E181" s="24">
+        <f t="shared" si="0"/>
+        <v>46323</v>
+      </c>
+      <c r="F181" s="12"/>
+    </row>
+    <row r="182" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B182" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C182" s="12">
+        <v>95</v>
+      </c>
+      <c r="D182" s="24">
+        <v>46309</v>
+      </c>
+      <c r="E182" s="24">
+        <f t="shared" si="0"/>
+        <v>46324</v>
+      </c>
+      <c r="F182" s="12"/>
+    </row>
+    <row r="183" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B183" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C183" s="12">
+        <v>64</v>
+      </c>
+      <c r="D183" s="24">
+        <v>46318</v>
+      </c>
+      <c r="E183" s="24">
+        <f t="shared" si="0"/>
+        <v>46333</v>
+      </c>
+      <c r="F183" s="12"/>
+    </row>
+    <row r="184" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B184" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C184" s="12">
+        <v>10</v>
+      </c>
+      <c r="D184" s="24">
+        <v>46301</v>
+      </c>
+      <c r="E184" s="24">
+        <f t="shared" si="0"/>
+        <v>46316</v>
+      </c>
+      <c r="F184" s="12"/>
+    </row>
+    <row r="185" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B185" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C185" s="12">
+        <v>10</v>
+      </c>
+      <c r="D185" s="24">
+        <v>46307</v>
+      </c>
+      <c r="E185" s="24">
+        <f t="shared" si="0"/>
+        <v>46322</v>
+      </c>
+      <c r="F185" s="12"/>
+    </row>
+    <row r="186" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B186" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C186" s="12">
+        <v>37</v>
+      </c>
+      <c r="D186" s="24">
+        <v>46301</v>
+      </c>
+      <c r="E186" s="24">
+        <f t="shared" si="0"/>
+        <v>46316</v>
+      </c>
+      <c r="F186" s="12"/>
+    </row>
+    <row r="187" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B187" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C187" s="12">
+        <v>37</v>
+      </c>
+      <c r="D187" s="24">
+        <v>46307</v>
+      </c>
+      <c r="E187" s="24">
+        <f t="shared" si="0"/>
+        <v>46322</v>
+      </c>
+      <c r="F187" s="12"/>
+    </row>
+    <row r="188" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B188" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C188" s="12">
+        <v>1</v>
+      </c>
+      <c r="D188" s="24">
+        <v>46314</v>
+      </c>
+      <c r="E188" s="24">
+        <f t="shared" si="0"/>
+        <v>46329</v>
+      </c>
+      <c r="F188" s="12"/>
+    </row>
+    <row r="189" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B189" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C189" s="12">
+        <v>30</v>
+      </c>
+      <c r="D189" s="24">
+        <v>46321</v>
+      </c>
+      <c r="E189" s="24">
+        <f t="shared" si="0"/>
+        <v>46336</v>
+      </c>
+      <c r="F189" s="12"/>
+    </row>
+    <row r="190" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B190" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C190" s="12">
+        <v>9</v>
+      </c>
+      <c r="D190" s="24">
+        <v>46301</v>
+      </c>
+      <c r="E190" s="24">
+        <f t="shared" si="0"/>
+        <v>46316</v>
+      </c>
+      <c r="F190" s="12"/>
+    </row>
+    <row r="191" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B191" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C191" s="12">
+        <v>5</v>
+      </c>
+      <c r="D191" s="24">
+        <v>46307</v>
+      </c>
+      <c r="E191" s="24">
+        <f t="shared" si="0"/>
+        <v>46322</v>
+      </c>
+      <c r="F191" s="12"/>
+    </row>
+    <row r="192" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B192" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C192" s="12">
+        <v>9</v>
+      </c>
+      <c r="D192" s="24">
+        <v>46321</v>
+      </c>
+      <c r="E192" s="24">
+        <f t="shared" si="0"/>
+        <v>46336</v>
+      </c>
+      <c r="F192" s="12"/>
+    </row>
+    <row r="193" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B193" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C193" s="12">
+        <v>31</v>
+      </c>
+      <c r="D193" s="24">
+        <v>46321</v>
+      </c>
+      <c r="E193" s="24">
+        <f t="shared" si="0"/>
+        <v>46336</v>
+      </c>
+      <c r="F193" s="12"/>
+    </row>
+    <row r="194" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B194" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C194" s="12">
+        <v>11</v>
+      </c>
+      <c r="D194" s="24">
+        <v>46318</v>
+      </c>
+      <c r="E194" s="24">
+        <f t="shared" si="0"/>
+        <v>46333</v>
+      </c>
+      <c r="F194" s="12"/>
+    </row>
+    <row r="195" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B195" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C195" s="12">
+        <v>19</v>
+      </c>
+      <c r="D195" s="24">
+        <v>46321</v>
+      </c>
+      <c r="E195" s="24">
+        <f t="shared" si="0"/>
+        <v>46336</v>
+      </c>
+      <c r="F195" s="12"/>
+    </row>
+    <row r="196" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B196" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C196" s="12">
+        <v>14</v>
+      </c>
+      <c r="D196" s="24">
+        <v>46301</v>
+      </c>
+      <c r="E196" s="24">
+        <f t="shared" si="0"/>
+        <v>46316</v>
+      </c>
+      <c r="F196" s="12"/>
+    </row>
+    <row r="197" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B197" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C197" s="12">
+        <v>9</v>
+      </c>
+      <c r="D197" s="24">
+        <v>46307</v>
+      </c>
+      <c r="E197" s="24">
+        <f t="shared" si="0"/>
+        <v>46322</v>
+      </c>
+      <c r="F197" s="12"/>
+    </row>
+    <row r="198" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B198" s="41"/>
+      <c r="C198" s="12"/>
+      <c r="D198" s="24"/>
+      <c r="E198" s="24"/>
+      <c r="F198" s="12"/>
+    </row>
+    <row r="199" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B199" s="41"/>
+      <c r="C199" s="12"/>
+      <c r="D199" s="24"/>
+      <c r="E199" s="24"/>
+      <c r="F199" s="12"/>
+    </row>
+    <row r="200" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B200" s="12"/>
+      <c r="C200" s="42"/>
+      <c r="D200" s="24"/>
+      <c r="E200" s="24"/>
+      <c r="F200" s="12"/>
+    </row>
+    <row r="201" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B201" s="12"/>
+      <c r="C201" s="12"/>
+      <c r="D201" s="24"/>
+      <c r="E201" s="24"/>
+      <c r="F201" s="12"/>
+    </row>
+    <row r="202" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B202" s="43"/>
+      <c r="C202" s="42"/>
+      <c r="D202" s="24"/>
+      <c r="E202" s="24"/>
+      <c r="F202" s="12"/>
+    </row>
+    <row r="203" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B203" s="12"/>
+      <c r="C203" s="12"/>
+      <c r="D203" s="24"/>
+      <c r="E203" s="24"/>
+      <c r="F203" s="12"/>
+    </row>
+    <row r="204" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B204" s="12"/>
+      <c r="C204" s="12"/>
+      <c r="D204" s="24"/>
+      <c r="E204" s="24"/>
+      <c r="F204" s="12"/>
+    </row>
+    <row r="205" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B205" s="43"/>
+      <c r="C205" s="42"/>
+      <c r="D205" s="24"/>
+      <c r="E205" s="24"/>
+      <c r="F205" s="12"/>
+    </row>
+    <row r="206" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B206" s="41"/>
+      <c r="C206" s="13"/>
+      <c r="D206" s="24"/>
+      <c r="E206" s="24"/>
+      <c r="F206" s="12"/>
+    </row>
+    <row r="207" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B207" s="12"/>
+      <c r="C207" s="42"/>
+      <c r="D207" s="24"/>
+      <c r="E207" s="24"/>
+      <c r="F207" s="12"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B1:E172" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="B1:F1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3810,33 +4345,33 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A4:L10"/>
+  <dimension ref="A4:P10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="39" t="s">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
-    </row>
-    <row r="5" spans="1:12" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
+      <c r="K4" s="40"/>
+      <c r="L4" s="40"/>
+    </row>
+    <row r="5" spans="1:16" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G5" s="34"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>1</v>
       </c>
@@ -3873,8 +4408,20 @@
       <c r="L6" s="13" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="N6" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="O6" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="P6" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>13</v>
       </c>
@@ -3893,8 +4440,12 @@
       <c r="J7" s="13"/>
       <c r="K7" s="13"/>
       <c r="L7" s="13"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="13"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>20</v>
       </c>
@@ -3913,8 +4464,12 @@
       <c r="J8" s="13"/>
       <c r="K8" s="13"/>
       <c r="L8" s="13"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M8" s="13"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>35</v>
       </c>
@@ -3933,8 +4488,12 @@
       <c r="J9" s="13"/>
       <c r="K9" s="13"/>
       <c r="L9" s="13"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M9" s="13"/>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="13"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>14</v>
       </c>
@@ -3957,26 +4516,33 @@
         <v>124</v>
       </c>
       <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13">
+        <v>100</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A4:L4"/>
   </mergeCells>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A4:L8"/>
+  <dimension ref="A4:P8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -4013,8 +4579,20 @@
       <c r="L6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6" s="39" t="s">
+        <v>84</v>
+      </c>
+      <c r="N6" s="39" t="s">
+        <v>85</v>
+      </c>
+      <c r="O6" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="P6" s="39" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4022,7 +4600,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -4035,8 +4613,12 @@
       <c r="J8">
         <v>113</v>
       </c>
+      <c r="P8">
+        <v>80</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>